<commit_message>
add test data, update unit tests accordingly
</commit_message>
<xml_diff>
--- a/src/test/resources/testobjectmodeldefinition.xlsx
+++ b/src/test/resources/testobjectmodeldefinition.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin/stuff/objectmodeldiagramgenerator/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DD609D-529F-0649-8BAF-A291B432290E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F2F8E5-08D3-A74C-B390-C04739FB5BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="23500" activeTab="1" xr2:uid="{EA4244F2-FE33-7643-A566-43DD5B4E5092}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="businessevents" sheetId="25" r:id="rId3"/>
     <sheet name="oms_PersonsAndHouses_state1" sheetId="26" r:id="rId4"/>
     <sheet name="oms_PersonsAndHouses_state2" sheetId="27" r:id="rId5"/>
+    <sheet name="___oms_Persons_state1" sheetId="28" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="125">
   <si>
     <t>name</t>
   </si>
@@ -351,13 +352,73 @@
   </si>
   <si>
     <t>scenario1, scenario3, scenario4</t>
+  </si>
+  <si>
+    <t>scenario6</t>
+  </si>
+  <si>
+    <t>Anton, Berta, and Charlie become friends and get older.</t>
+  </si>
+  <si>
+    <t>event0601</t>
+  </si>
+  <si>
+    <t>Berta and Charlie become friends.</t>
+  </si>
+  <si>
+    <t>event0602</t>
+  </si>
+  <si>
+    <t>event0603</t>
+  </si>
+  <si>
+    <t>event0604</t>
+  </si>
+  <si>
+    <t>Anton joins Berta and Charlie's friendship.</t>
+  </si>
+  <si>
+    <t>Anton and Charlie get one year older.</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>p2p02</t>
+  </si>
+  <si>
+    <t>friendship</t>
+  </si>
+  <si>
+    <t>(berta, charlie)</t>
+  </si>
+  <si>
+    <t>scenario1, scenario2, scenario4</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>(anton, berta, charlie)</t>
+  </si>
+  <si>
+    <t>event0605</t>
+  </si>
+  <si>
+    <t>Anton and Berta get divorced.</t>
+  </si>
+  <si>
+    <t>After Anton, Berta, and Charlie celebrated a party, Anton and Charlie are not friends anymore.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -391,8 +452,14 @@
       <name val="Consolas"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -415,6 +482,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -547,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -592,6 +665,9 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -613,11 +689,67 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -884,12 +1016,12 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F5B660FE-5499-6D4F-B192-6D495D38DF3B}" name="Tabelle17" displayName="Tabelle17" ref="A1:C17" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:C17" xr:uid="{422A6A28-4F84-CA4D-BC76-24F29CBA51D2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F5B660FE-5499-6D4F-B192-6D495D38DF3B}" name="Tabelle17" displayName="Tabelle17" ref="A1:C23" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A1:C23" xr:uid="{422A6A28-4F84-CA4D-BC76-24F29CBA51D2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{938701D0-9835-4745-A220-8C6068F221FF}" name="Key" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{381D88C7-4F57-284F-9F9B-E9AEB9E0E9F8}" name="Description" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{0A673B68-A98A-1B41-889D-06C26B97C1F1}" name="ScenarioKey" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{938701D0-9835-4745-A220-8C6068F221FF}" name="Key" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{381D88C7-4F57-284F-9F9B-E9AEB9E0E9F8}" name="Description" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{0A673B68-A98A-1B41-889D-06C26B97C1F1}" name="ScenarioKey" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1253,7 +1385,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F5FAD2-8154-0D49-A79A-D1DF14B91F10}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1325,6 +1457,17 @@
       </c>
       <c r="C10" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1339,11 +1482,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{223ACBB0-66D3-934A-A293-379036E0F203}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" style="3" customWidth="1"/>
-    <col min="2" max="2" width="93.1640625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="96.6640625" style="7" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" style="7" customWidth="1"/>
     <col min="4" max="16384" width="11" style="5"/>
   </cols>
@@ -1509,6 +1652,66 @@
       </c>
       <c r="C17" s="9" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="4"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="8"/>
+    </row>
+    <row r="19" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A23" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1543,66 +1746,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="21" t="s">
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="22" t="s">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22" t="s">
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="15" t="s">
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15" t="s">
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="19"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="20"/>
       <c r="C3" s="10" t="s">
         <v>46</v>
       </c>
@@ -3010,22 +3213,22 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="S8:XFD21 P22:XFD24 A4:R24 A25:XFD1048576">
-    <cfRule type="containsBlanks" dxfId="7" priority="3" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="11" priority="3" stopIfTrue="1">
       <formula>LEN(TRIM(A4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S8:XFD21 P22:XFD24 C4:R24 C25:XFD1048576">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="notEqual">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:XFD7">
-    <cfRule type="containsBlanks" dxfId="5" priority="1" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="9" priority="1" stopIfTrue="1">
       <formula>LEN(TRIM(S1))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:XFD7">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="notEqual">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3058,66 +3261,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="21" t="s">
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="22" t="s">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22" t="s">
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="15" t="s">
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15" t="s">
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15" t="s">
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="19"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="20"/>
       <c r="C3" s="10" t="s">
         <v>46</v>
       </c>
@@ -3236,22 +3439,22 @@
     <mergeCell ref="P2:R2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:R4 A5:XFD1048576">
-    <cfRule type="containsBlanks" dxfId="3" priority="3" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="7" priority="3" stopIfTrue="1">
       <formula>LEN(TRIM(A4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:R4 C5:XFD1048576">
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="notEqual">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:XFD4">
-    <cfRule type="containsBlanks" dxfId="1" priority="1" stopIfTrue="1">
+    <cfRule type="containsBlanks" dxfId="5" priority="1" stopIfTrue="1">
       <formula>LEN(TRIM(S1))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:XFD4">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="notEqual">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="notEqual">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3259,13 +3462,242 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5D323E-2665-E041-95E7-E289DAEFE0FA}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="3" max="5" width="10.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+    </row>
+    <row r="2" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+    </row>
+    <row r="3" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="19"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="H4" s="25" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="A4:E4 A5:XFD1048576">
+    <cfRule type="containsBlanks" dxfId="3" priority="3" stopIfTrue="1">
+      <formula>LEN(TRIM(A4))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:E4 C5:XFD1048576">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="notEqual">
+      <formula>"-"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I1:XFD4">
+    <cfRule type="containsBlanks" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>LEN(TRIM(I1))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I1:XFD4">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="notEqual">
+      <formula>"-"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E5:E6" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3427,15 +3859,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44EA3924-C60D-4AB3-8333-F249729C0DDD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2124C44-2049-4194-ADAF-B2DF55B36692}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="fe6e65e6-3f48-4872-a1e7-e48555659f5f"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3459,17 +3902,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2124C44-2049-4194-ADAF-B2DF55B36692}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44EA3924-C60D-4AB3-8333-F249729C0DDD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="fe6e65e6-3f48-4872-a1e7-e48555659f5f"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add test diagrams for scenario6, unit tests fail!
</commit_message>
<xml_diff>
--- a/src/test/resources/testobjectmodeldefinition.xlsx
+++ b/src/test/resources/testobjectmodeldefinition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin/stuff/objectmodeldiagramgenerator/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F2F8E5-08D3-A74C-B390-C04739FB5BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D80C7D-93E4-284E-844C-F5944F20EA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="23500" activeTab="1" xr2:uid="{EA4244F2-FE33-7643-A566-43DD5B4E5092}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="businessevents" sheetId="25" r:id="rId3"/>
     <sheet name="oms_PersonsAndHouses_state1" sheetId="26" r:id="rId4"/>
     <sheet name="oms_PersonsAndHouses_state2" sheetId="27" r:id="rId5"/>
-    <sheet name="___oms_Persons_state1" sheetId="28" r:id="rId6"/>
+    <sheet name="oms_Persons_state1" sheetId="28" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="127">
   <si>
     <t>name</t>
   </si>
@@ -357,9 +357,6 @@
     <t>scenario6</t>
   </si>
   <si>
-    <t>Anton, Berta, and Charlie become friends and get older.</t>
-  </si>
-  <si>
     <t>event0601</t>
   </si>
   <si>
@@ -411,7 +408,16 @@
     <t>Anton and Berta get divorced.</t>
   </si>
   <si>
-    <t>After Anton, Berta, and Charlie celebrated a party, Anton and Charlie are not friends anymore.</t>
+    <t>predivorce</t>
+  </si>
+  <si>
+    <t>(anton, charlie)</t>
+  </si>
+  <si>
+    <t>After Anton, Berta, and Charlie celebrated a party, Berta leaves the friendship.</t>
+  </si>
+  <si>
+    <t>Anton, Berta, and Charlie become friends and get older. Then the situation changes again.</t>
   </si>
 </sst>
 </file>
@@ -665,6 +671,12 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -687,12 +699,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1464,10 +1470,10 @@
         <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1661,56 +1667,56 @@
     </row>
     <row r="19" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="16" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" s="16" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C22" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="16" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="16" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1746,66 +1752,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="22" t="s">
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="23" t="s">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23" t="s">
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="16" t="s">
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16" t="s">
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16" t="s">
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
     </row>
     <row r="3" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19"/>
-      <c r="B3" s="20"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="10" t="s">
         <v>46</v>
       </c>
@@ -3261,66 +3267,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="22" t="s">
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="23" t="s">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23" t="s">
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="16" t="s">
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="16" t="s">
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16" t="s">
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
     </row>
     <row r="3" spans="1:18" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19"/>
-      <c r="B3" s="20"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="10" t="s">
         <v>46</v>
       </c>
@@ -3464,51 +3470,51 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B5D323E-2665-E041-95E7-E289DAEFE0FA}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1"/>
     <col min="3" max="5" width="10.83203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="8.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="20.5" style="1" customWidth="1"/>
     <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="16" t="s">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16" t="s">
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="1:8" s="2" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19"/>
-      <c r="B3" s="20"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="15" t="s">
         <v>58</v>
       </c>
@@ -3530,7 +3536,7 @@
     </row>
     <row r="4" spans="1:8" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
@@ -3544,22 +3550,22 @@
       <c r="E4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="G4" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="H4" s="17" t="s">
         <v>116</v>
-      </c>
-      <c r="H4" s="25" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>97</v>
@@ -3568,7 +3574,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>1</v>
@@ -3582,10 +3588,10 @@
     </row>
     <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>99</v>
@@ -3594,7 +3600,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>1</v>
@@ -3608,54 +3614,106 @@
     </row>
     <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="G7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="G8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>117</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3695,9 +3753,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3859,26 +3920,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2124C44-2049-4194-ADAF-B2DF55B36692}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44EA3924-C60D-4AB3-8333-F249729C0DDD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="fe6e65e6-3f48-4872-a1e7-e48555659f5f"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3902,9 +3952,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44EA3924-C60D-4AB3-8333-F249729C0DDD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2124C44-2049-4194-ADAF-B2DF55B36692}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="fe6e65e6-3f48-4872-a1e7-e48555659f5f"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>